<commit_message>
Amazon scraper checkpoint: Men'S Ethnic Shoes
</commit_message>
<xml_diff>
--- a/output/Amazon_Seller_Master_Data.xlsx
+++ b/output/Amazon_Seller_Master_Data.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Amazon Sellers" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Amazon Sellers'!$A$1:$U$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Amazon Sellers'!$A$1:$U$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,13 +460,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U6"/>
+  <dimension ref="A1:U9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="31" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
@@ -696,7 +696,7 @@
           <t>Men'S Slippers &amp; Flip Flops</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr"/>
+      <c r="B3" s="2" t="n"/>
       <c r="C3" s="3" t="n">
         <v>1</v>
       </c>
@@ -750,7 +750,7 @@
           <t>19176 hall road, suite 130</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr"/>
+      <c r="N3" s="2" t="n"/>
       <c r="O3" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -793,7 +793,7 @@
           <t>Men'S Slippers &amp; Flip Flops</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr"/>
+      <c r="B4" s="2" t="n"/>
       <c r="C4" s="3" t="n">
         <v>2</v>
       </c>
@@ -847,7 +847,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="n"/>
       <c r="O4" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -890,7 +890,7 @@
           <t>Men'S Slippers &amp; Flip Flops</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr"/>
+      <c r="B5" s="2" t="n"/>
       <c r="C5" s="3" t="n">
         <v>3</v>
       </c>
@@ -944,7 +944,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr"/>
+      <c r="N5" s="2" t="n"/>
       <c r="O5" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -987,7 +987,7 @@
           <t>Men'S Slippers &amp; Flip Flops</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr"/>
+      <c r="B6" s="2" t="n"/>
       <c r="C6" s="3" t="n">
         <v>4</v>
       </c>
@@ -1041,7 +1041,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr"/>
+      <c r="N6" s="2" t="n"/>
       <c r="O6" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -1073,13 +1073,304 @@
         </is>
       </c>
       <c r="U6" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Men'S Ethnic Shoes</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr"/>
+      <c r="C7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Indian Classy Wear</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Men'S Ethnic Shoes</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M7" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr"/>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q7" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R7" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S7" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="T7" s="2" t="inlineStr">
+        <is>
+          <t>Needs Review</t>
+        </is>
+      </c>
+      <c r="U7" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Men'S Ethnic Shoes</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr"/>
+      <c r="C8" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Fausto Luckystar</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Men'S Ethnic Shoes</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>nhcwebmaster@noaa.gov</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr"/>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q8" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R8" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S8" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="T8" s="2" t="inlineStr">
+        <is>
+          <t>Partially Verified</t>
+        </is>
+      </c>
+      <c r="U8" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Men'S Ethnic Shoes</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr"/>
+      <c r="C9" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Cocoblu Retail</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Men'S Ethnic Shoes</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>support@cardgames.io</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M9" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr"/>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q9" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R9" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S9" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="T9" s="2" t="inlineStr">
+        <is>
+          <t>Partially Verified</t>
+        </is>
+      </c>
+      <c r="U9" s="2" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U6"/>
+  <autoFilter ref="A1:U9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Amazon scraper checkpoint: Men'S Clogs
</commit_message>
<xml_diff>
--- a/output/Amazon_Seller_Master_Data.xlsx
+++ b/output/Amazon_Seller_Master_Data.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Amazon Sellers" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Amazon Sellers'!$A$1:$U$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Amazon Sellers'!$A$1:$U$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U9"/>
+  <dimension ref="A1:U11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -1084,7 +1084,7 @@
           <t>Men'S Ethnic Shoes</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr"/>
+      <c r="B7" s="2" t="n"/>
       <c r="C7" s="3" t="n">
         <v>1</v>
       </c>
@@ -1138,7 +1138,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr"/>
+      <c r="N7" s="2" t="n"/>
       <c r="O7" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -1181,7 +1181,7 @@
           <t>Men'S Ethnic Shoes</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr"/>
+      <c r="B8" s="2" t="n"/>
       <c r="C8" s="3" t="n">
         <v>2</v>
       </c>
@@ -1235,7 +1235,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr"/>
+      <c r="N8" s="2" t="n"/>
       <c r="O8" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -1278,7 +1278,7 @@
           <t>Men'S Ethnic Shoes</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr"/>
+      <c r="B9" s="2" t="n"/>
       <c r="C9" s="3" t="n">
         <v>3</v>
       </c>
@@ -1332,7 +1332,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr"/>
+      <c r="N9" s="2" t="n"/>
       <c r="O9" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -1364,13 +1364,207 @@
         </is>
       </c>
       <c r="U9" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Men'S Clogs</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr"/>
+      <c r="C10" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Hike Store</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Men'S Clogs</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>info@hike-footwear.com</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M10" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr"/>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q10" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R10" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hikestore.com/</t>
+        </is>
+      </c>
+      <c r="T10" s="2" t="inlineStr">
+        <is>
+          <t>Partially Verified</t>
+        </is>
+      </c>
+      <c r="U10" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Men'S Clogs</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr"/>
+      <c r="C11" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>walkers shoes</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Men'S Clogs</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M11" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr"/>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q11" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R11" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S11" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="T11" s="2" t="inlineStr">
+        <is>
+          <t>Needs Review</t>
+        </is>
+      </c>
+      <c r="U11" s="2" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U9"/>
+  <autoFilter ref="A1:U11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Amazon scraper checkpoint: Boots
</commit_message>
<xml_diff>
--- a/output/Amazon_Seller_Master_Data.xlsx
+++ b/output/Amazon_Seller_Master_Data.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Amazon Sellers" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Amazon Sellers'!$A$1:$U$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Amazon Sellers'!$A$1:$U$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,13 +460,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U11"/>
+  <dimension ref="A1:U15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="31" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
@@ -477,7 +477,7 @@
     <col width="16" customWidth="1" min="12" max="12"/>
     <col width="39" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="21" customWidth="1" min="15" max="15"/>
     <col width="13" customWidth="1" min="16" max="16"/>
     <col width="13" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
@@ -1375,7 +1375,7 @@
           <t>Men'S Clogs</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr"/>
+      <c r="B10" s="2" t="n"/>
       <c r="C10" s="3" t="n">
         <v>1</v>
       </c>
@@ -1429,7 +1429,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="n"/>
       <c r="O10" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -1472,7 +1472,7 @@
           <t>Men'S Clogs</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr"/>
+      <c r="B11" s="2" t="n"/>
       <c r="C11" s="3" t="n">
         <v>2</v>
       </c>
@@ -1526,7 +1526,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr"/>
+      <c r="N11" s="2" t="n"/>
       <c r="O11" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -1558,13 +1558,401 @@
         </is>
       </c>
       <c r="U11" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Boots</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr"/>
+      <c r="C12" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Cocoblu Retail</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Boots</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>access@t-mobile.com</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M12" s="5" t="inlineStr">
+        <is>
+          <t>london &amp; partners, 169 union street, london se1 0ll. london &amp; partners is the growth agency for london. we are a social enterprise, combining purpose</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr"/>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>combining purpose</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q12" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R12" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S12" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="T12" s="2" t="inlineStr">
+        <is>
+          <t>Partially Verified</t>
+        </is>
+      </c>
+      <c r="U12" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Boots</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr"/>
+      <c r="C13" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>DADWANI'S FOOTWEAR PRIVATE LIMITED</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Boots</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>info@howmanyfps.com</t>
+        </is>
+      </c>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K13" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M13" s="5" t="inlineStr">
+        <is>
+          <t>450 longwater avenue, green park, reading, berkshire, rg2 6gf</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr"/>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>berkshire</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q13" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R13" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S13" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="T13" s="2" t="inlineStr">
+        <is>
+          <t>Partially Verified</t>
+        </is>
+      </c>
+      <c r="U13" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Boots</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr"/>
+      <c r="C14" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Do Bhai Bags &amp; Luggage</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Boots</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M14" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr"/>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q14" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R14" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S14" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="T14" s="2" t="inlineStr">
+        <is>
+          <t>Needs Review</t>
+        </is>
+      </c>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Boots</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr"/>
+      <c r="C15" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>KRAASA</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Boots</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>+916165581870</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M15" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr"/>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q15" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R15" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S15" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="T15" s="2" t="inlineStr">
+        <is>
+          <t>Partially Verified</t>
+        </is>
+      </c>
+      <c r="U15" s="2" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U11"/>
+  <autoFilter ref="A1:U15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Amazon scraper checkpoint: Sneakers
</commit_message>
<xml_diff>
--- a/output/Amazon_Seller_Master_Data.xlsx
+++ b/output/Amazon_Seller_Master_Data.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Amazon Sellers" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Amazon Sellers'!$A$1:$U$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Amazon Sellers'!$A$1:$U$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U17"/>
+  <dimension ref="A1:U22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -1860,7 +1860,7 @@
           <t>Men'S Clogs</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr"/>
+      <c r="B15" s="2" t="n"/>
       <c r="C15" s="3" t="n">
         <v>1</v>
       </c>
@@ -1914,7 +1914,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N15" s="2" t="inlineStr"/>
+      <c r="N15" s="2" t="n"/>
       <c r="O15" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -1957,7 +1957,7 @@
           <t>Men'S Clogs</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr"/>
+      <c r="B16" s="2" t="n"/>
       <c r="C16" s="3" t="n">
         <v>2</v>
       </c>
@@ -2011,7 +2011,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N16" s="2" t="inlineStr"/>
+      <c r="N16" s="2" t="n"/>
       <c r="O16" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -2054,7 +2054,7 @@
           <t>Men'S Clogs</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr"/>
+      <c r="B17" s="2" t="n"/>
       <c r="C17" s="3" t="n">
         <v>3</v>
       </c>
@@ -2108,7 +2108,7 @@
           <t>4700 s syracuse st #1050, denver, co 80237</t>
         </is>
       </c>
-      <c r="N17" s="2" t="inlineStr"/>
+      <c r="N17" s="2" t="n"/>
       <c r="O17" s="2" t="inlineStr">
         <is>
           <t>denver</t>
@@ -2140,13 +2140,498 @@
         </is>
       </c>
       <c r="U17" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Sneakers</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr"/>
+      <c r="C18" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Cocoblu Retail</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Sneakers</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>care@cocoblu.in</t>
+        </is>
+      </c>
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K18" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M18" s="5" t="inlineStr">
+        <is>
+          <t>6th floor, dlf centre, sansad marg, new delhi-110001</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr"/>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>new delhi</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="Q18" s="4" t="inlineStr">
+        <is>
+          <t>110001</t>
+        </is>
+      </c>
+      <c r="R18" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S18" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="T18" s="2" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="U18" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Sneakers</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr"/>
+      <c r="C19" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Asian Shoes</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Sneakers</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K19" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M19" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="inlineStr"/>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q19" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R19" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S19" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="T19" s="2" t="inlineStr">
+        <is>
+          <t>Needs Review</t>
+        </is>
+      </c>
+      <c r="U19" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Sneakers</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr"/>
+      <c r="C20" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Viraj Ent</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Sneakers</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>support@swimoutlet.com</t>
+        </is>
+      </c>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K20" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M20" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="inlineStr"/>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q20" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R20" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S20" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="T20" s="2" t="inlineStr">
+        <is>
+          <t>Partially Verified</t>
+        </is>
+      </c>
+      <c r="U20" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Sneakers</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr"/>
+      <c r="C21" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>APPOO TRADING</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Sneakers</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>sales@motorsport.com</t>
+        </is>
+      </c>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M21" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="inlineStr"/>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q21" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R21" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S21" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="T21" s="2" t="inlineStr">
+        <is>
+          <t>Partially Verified</t>
+        </is>
+      </c>
+      <c r="U21" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Sneakers</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr"/>
+      <c r="C22" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>BansalEnterprises</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Sneakers</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>contact@kiricard.com</t>
+        </is>
+      </c>
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M22" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr"/>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q22" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R22" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S22" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="T22" s="2" t="inlineStr">
+        <is>
+          <t>Partially Verified</t>
+        </is>
+      </c>
+      <c r="U22" s="2" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U17"/>
+  <autoFilter ref="A1:U22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Amazon scraper checkpoint: Women'S Flats
</commit_message>
<xml_diff>
--- a/output/Amazon_Seller_Master_Data.xlsx
+++ b/output/Amazon_Seller_Master_Data.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Amazon Sellers" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Amazon Sellers'!$A$1:$U$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Amazon Sellers'!$A$1:$U$24</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U22"/>
+  <dimension ref="A1:U24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -471,7 +471,7 @@
     <col width="31" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
     <col width="17" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="33" customWidth="1" min="9" max="9"/>
     <col width="19" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
@@ -2151,7 +2151,7 @@
           <t>Sneakers</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr"/>
+      <c r="B18" s="2" t="n"/>
       <c r="C18" s="3" t="n">
         <v>1</v>
       </c>
@@ -2205,7 +2205,7 @@
           <t>6th floor, dlf centre, sansad marg, new delhi-110001</t>
         </is>
       </c>
-      <c r="N18" s="2" t="inlineStr"/>
+      <c r="N18" s="2" t="n"/>
       <c r="O18" s="2" t="inlineStr">
         <is>
           <t>new delhi</t>
@@ -2248,7 +2248,7 @@
           <t>Sneakers</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr"/>
+      <c r="B19" s="2" t="n"/>
       <c r="C19" s="3" t="n">
         <v>2</v>
       </c>
@@ -2302,7 +2302,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N19" s="2" t="inlineStr"/>
+      <c r="N19" s="2" t="n"/>
       <c r="O19" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -2345,7 +2345,7 @@
           <t>Sneakers</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr"/>
+      <c r="B20" s="2" t="n"/>
       <c r="C20" s="3" t="n">
         <v>3</v>
       </c>
@@ -2399,7 +2399,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N20" s="2" t="inlineStr"/>
+      <c r="N20" s="2" t="n"/>
       <c r="O20" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -2442,7 +2442,7 @@
           <t>Sneakers</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr"/>
+      <c r="B21" s="2" t="n"/>
       <c r="C21" s="3" t="n">
         <v>4</v>
       </c>
@@ -2496,7 +2496,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N21" s="2" t="inlineStr"/>
+      <c r="N21" s="2" t="n"/>
       <c r="O21" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -2539,7 +2539,7 @@
           <t>Sneakers</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr"/>
+      <c r="B22" s="2" t="n"/>
       <c r="C22" s="3" t="n">
         <v>5</v>
       </c>
@@ -2593,7 +2593,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N22" s="2" t="inlineStr"/>
+      <c r="N22" s="2" t="n"/>
       <c r="O22" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -2625,13 +2625,207 @@
         </is>
       </c>
       <c r="U22" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Women'S Flats</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr"/>
+      <c r="C23" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>FashionVillage20</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Women'S Flats</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>contact@axis-intelligence.com</t>
+        </is>
+      </c>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M23" s="5" t="inlineStr">
+        <is>
+          <t>200 w. oak street, first floor, fort collins, co 80521</t>
+        </is>
+      </c>
+      <c r="N23" s="2" t="inlineStr"/>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>fort collins</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q23" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R23" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S23" s="2" t="inlineStr">
+        <is>
+          <t>https://fashionville.com/</t>
+        </is>
+      </c>
+      <c r="T23" s="2" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="U23" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Women'S Flats</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr"/>
+      <c r="C24" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>AnKaHu Enterprises</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Women'S Flats</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>info@worldmetrics.org</t>
+        </is>
+      </c>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M24" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="inlineStr"/>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q24" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R24" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S24" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="T24" s="2" t="inlineStr">
+        <is>
+          <t>Partially Verified</t>
+        </is>
+      </c>
+      <c r="U24" s="2" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U22"/>
+  <autoFilter ref="A1:U24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Amazon scraper checkpoint: Women'S Heels
</commit_message>
<xml_diff>
--- a/output/Amazon_Seller_Master_Data.xlsx
+++ b/output/Amazon_Seller_Master_Data.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Amazon Sellers" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Amazon Sellers'!$A$1:$U$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Amazon Sellers'!$A$1:$U$27</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U24"/>
+  <dimension ref="A1:U27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -2636,7 +2636,7 @@
           <t>Women'S Flats</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr"/>
+      <c r="B23" s="2" t="n"/>
       <c r="C23" s="3" t="n">
         <v>1</v>
       </c>
@@ -2690,7 +2690,7 @@
           <t>200 w. oak street, first floor, fort collins, co 80521</t>
         </is>
       </c>
-      <c r="N23" s="2" t="inlineStr"/>
+      <c r="N23" s="2" t="n"/>
       <c r="O23" s="2" t="inlineStr">
         <is>
           <t>fort collins</t>
@@ -2733,7 +2733,7 @@
           <t>Women'S Flats</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr"/>
+      <c r="B24" s="2" t="n"/>
       <c r="C24" s="3" t="n">
         <v>2</v>
       </c>
@@ -2787,7 +2787,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N24" s="2" t="inlineStr"/>
+      <c r="N24" s="2" t="n"/>
       <c r="O24" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -2819,13 +2819,304 @@
         </is>
       </c>
       <c r="U24" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Women'S Heels</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr"/>
+      <c r="C25" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>JM LOOKS</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Women'S Heels</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>+918178788820</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>support@jmlooks.com</t>
+        </is>
+      </c>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K25" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M25" s="5" t="inlineStr">
+        <is>
+          <t>Basement Floor, Jm Looks, Pillar No.463, 73/7/3</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr"/>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>Jm Looks</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q25" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R25" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.jmlooks.com/</t>
+        </is>
+      </c>
+      <c r="T25" s="2" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="U25" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Women'S Heels</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr"/>
+      <c r="C26" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Cocoblu Retail</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Women'S Heels</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>info@discovertheworld.com</t>
+        </is>
+      </c>
+      <c r="J26" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M26" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr"/>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q26" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R26" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S26" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="T26" s="2" t="inlineStr">
+        <is>
+          <t>Partially Verified</t>
+        </is>
+      </c>
+      <c r="U26" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Women'S Heels</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr"/>
+      <c r="C27" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Do Bhai Bags &amp; Luggage</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Women'S Heels</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="J27" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K27" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M27" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="inlineStr"/>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q27" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R27" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S27" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="T27" s="2" t="inlineStr">
+        <is>
+          <t>Needs Review</t>
+        </is>
+      </c>
+      <c r="U27" s="2" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U24"/>
+  <autoFilter ref="A1:U27"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Amazon scraper checkpoint: Women'S Casual Shoes
</commit_message>
<xml_diff>
--- a/output/Amazon_Seller_Master_Data.xlsx
+++ b/output/Amazon_Seller_Master_Data.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Amazon Sellers" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Amazon Sellers'!$A$1:$U$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Amazon Sellers'!$A$1:$U$32</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U27"/>
+  <dimension ref="A1:U32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -471,7 +471,7 @@
     <col width="31" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
     <col width="17" customWidth="1" min="8" max="8"/>
-    <col width="33" customWidth="1" min="9" max="9"/>
+    <col width="35" customWidth="1" min="9" max="9"/>
     <col width="19" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
@@ -481,7 +481,7 @@
     <col width="17" customWidth="1" min="16" max="16"/>
     <col width="13" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
-    <col width="37" customWidth="1" min="19" max="19"/>
+    <col width="38" customWidth="1" min="19" max="19"/>
     <col width="22" customWidth="1" min="20" max="20"/>
     <col width="12" customWidth="1" min="21" max="21"/>
   </cols>
@@ -2830,7 +2830,7 @@
           <t>Women'S Heels</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr"/>
+      <c r="B25" s="2" t="n"/>
       <c r="C25" s="3" t="n">
         <v>1</v>
       </c>
@@ -2884,7 +2884,7 @@
           <t>Basement Floor, Jm Looks, Pillar No.463, 73/7/3</t>
         </is>
       </c>
-      <c r="N25" s="2" t="inlineStr"/>
+      <c r="N25" s="2" t="n"/>
       <c r="O25" s="2" t="inlineStr">
         <is>
           <t>Jm Looks</t>
@@ -2927,7 +2927,7 @@
           <t>Women'S Heels</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr"/>
+      <c r="B26" s="2" t="n"/>
       <c r="C26" s="3" t="n">
         <v>2</v>
       </c>
@@ -2981,7 +2981,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N26" s="2" t="inlineStr"/>
+      <c r="N26" s="2" t="n"/>
       <c r="O26" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -3024,7 +3024,7 @@
           <t>Women'S Heels</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr"/>
+      <c r="B27" s="2" t="n"/>
       <c r="C27" s="3" t="n">
         <v>3</v>
       </c>
@@ -3078,7 +3078,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N27" s="2" t="inlineStr"/>
+      <c r="N27" s="2" t="n"/>
       <c r="O27" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -3110,13 +3110,498 @@
         </is>
       </c>
       <c r="U27" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Women'S Casual Shoes</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr"/>
+      <c r="C28" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Cocoblu Retail</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Women'S Casual Shoes</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>care@cocoblu.in</t>
+        </is>
+      </c>
+      <c r="J28" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K28" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M28" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr"/>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q28" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R28" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cocoblu.in/</t>
+        </is>
+      </c>
+      <c r="T28" s="2" t="inlineStr">
+        <is>
+          <t>Partially Verified</t>
+        </is>
+      </c>
+      <c r="U28" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Women'S Casual Shoes</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr"/>
+      <c r="C29" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Viraj Ent</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Women'S Casual Shoes</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="J29" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K29" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L29" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M29" s="5" t="inlineStr">
+        <is>
+          <t>3472 olney laytonsville road, olney, md 20832</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr"/>
+      <c r="O29" s="2" t="inlineStr">
+        <is>
+          <t>olney</t>
+        </is>
+      </c>
+      <c r="P29" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q29" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R29" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S29" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="T29" s="2" t="inlineStr">
+        <is>
+          <t>Partially Verified</t>
+        </is>
+      </c>
+      <c r="U29" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Women'S Casual Shoes</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr"/>
+      <c r="C30" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>BansalEnterprises</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Women'S Casual Shoes</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>bk5671@caveenterprises.com</t>
+        </is>
+      </c>
+      <c r="J30" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K30" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L30" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M30" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="inlineStr"/>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q30" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R30" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bansalenterprises.com/</t>
+        </is>
+      </c>
+      <c r="T30" s="2" t="inlineStr">
+        <is>
+          <t>Partially Verified</t>
+        </is>
+      </c>
+      <c r="U30" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Women'S Casual Shoes</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr"/>
+      <c r="C31" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>RELAXO FOOTWEARS LIMITED</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Women'S Casual Shoes</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>customercare@relaxofootwear.com</t>
+        </is>
+      </c>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K31" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M31" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr"/>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P31" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q31" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R31" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S31" s="2" t="inlineStr">
+        <is>
+          <t>https://relaxofootwear.com/</t>
+        </is>
+      </c>
+      <c r="T31" s="2" t="inlineStr">
+        <is>
+          <t>Partially Verified</t>
+        </is>
+      </c>
+      <c r="U31" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Women'S Casual Shoes</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr"/>
+      <c r="C32" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Bata_India Ltd</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Women'S Casual Shoes</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>+919797888868</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="J32" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K32" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L32" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M32" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="inlineStr"/>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P32" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q32" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R32" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S32" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="T32" s="2" t="inlineStr">
+        <is>
+          <t>Partially Verified</t>
+        </is>
+      </c>
+      <c r="U32" s="2" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U27"/>
+  <autoFilter ref="A1:U32"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Amazon scraper checkpoint: Women'S Formals
</commit_message>
<xml_diff>
--- a/output/Amazon_Seller_Master_Data.xlsx
+++ b/output/Amazon_Seller_Master_Data.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Amazon Sellers" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Amazon Sellers'!$A$1:$U$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Amazon Sellers'!$A$1:$U$35</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U32"/>
+  <dimension ref="A1:U35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -471,7 +471,7 @@
     <col width="31" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
     <col width="17" customWidth="1" min="8" max="8"/>
-    <col width="35" customWidth="1" min="9" max="9"/>
+    <col width="37" customWidth="1" min="9" max="9"/>
     <col width="19" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
@@ -3121,7 +3121,7 @@
           <t>Women'S Casual Shoes</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr"/>
+      <c r="B28" s="2" t="n"/>
       <c r="C28" s="3" t="n">
         <v>1</v>
       </c>
@@ -3175,7 +3175,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N28" s="2" t="inlineStr"/>
+      <c r="N28" s="2" t="n"/>
       <c r="O28" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -3218,7 +3218,7 @@
           <t>Women'S Casual Shoes</t>
         </is>
       </c>
-      <c r="B29" s="2" t="inlineStr"/>
+      <c r="B29" s="2" t="n"/>
       <c r="C29" s="3" t="n">
         <v>2</v>
       </c>
@@ -3272,7 +3272,7 @@
           <t>3472 olney laytonsville road, olney, md 20832</t>
         </is>
       </c>
-      <c r="N29" s="2" t="inlineStr"/>
+      <c r="N29" s="2" t="n"/>
       <c r="O29" s="2" t="inlineStr">
         <is>
           <t>olney</t>
@@ -3315,7 +3315,7 @@
           <t>Women'S Casual Shoes</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr"/>
+      <c r="B30" s="2" t="n"/>
       <c r="C30" s="3" t="n">
         <v>3</v>
       </c>
@@ -3369,7 +3369,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N30" s="2" t="inlineStr"/>
+      <c r="N30" s="2" t="n"/>
       <c r="O30" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -3412,7 +3412,7 @@
           <t>Women'S Casual Shoes</t>
         </is>
       </c>
-      <c r="B31" s="2" t="inlineStr"/>
+      <c r="B31" s="2" t="n"/>
       <c r="C31" s="3" t="n">
         <v>4</v>
       </c>
@@ -3466,7 +3466,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N31" s="2" t="inlineStr"/>
+      <c r="N31" s="2" t="n"/>
       <c r="O31" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -3509,7 +3509,7 @@
           <t>Women'S Casual Shoes</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr"/>
+      <c r="B32" s="2" t="n"/>
       <c r="C32" s="3" t="n">
         <v>5</v>
       </c>
@@ -3563,7 +3563,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N32" s="2" t="inlineStr"/>
+      <c r="N32" s="2" t="n"/>
       <c r="O32" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -3595,13 +3595,304 @@
         </is>
       </c>
       <c r="U32" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Women'S Formals</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr"/>
+      <c r="C33" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Cocoblu Retail</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Women'S Formals</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>care@cocoblu.in</t>
+        </is>
+      </c>
+      <c r="J33" s="4" t="inlineStr">
+        <is>
+          <t>29AAJCC8517E1ZH</t>
+        </is>
+      </c>
+      <c r="K33" s="4" t="inlineStr">
+        <is>
+          <t>AAJCC8517E</t>
+        </is>
+      </c>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M33" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="inlineStr"/>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P33" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q33" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R33" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cocoblu.in/</t>
+        </is>
+      </c>
+      <c r="T33" s="2" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="U33" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Women'S Formals</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr"/>
+      <c r="C34" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Brinda Enterpris</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Women'S Formals</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>info@svsvet.com</t>
+        </is>
+      </c>
+      <c r="J34" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K34" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L34" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M34" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="inlineStr"/>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P34" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q34" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R34" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S34" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="T34" s="2" t="inlineStr">
+        <is>
+          <t>Partially Verified</t>
+        </is>
+      </c>
+      <c r="U34" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Women'S Formals</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr"/>
+      <c r="C35" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>LABHU BAA EMPORIO</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Women'S Formals</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>propertymanager@summerplaceal.com</t>
+        </is>
+      </c>
+      <c r="J35" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K35" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M35" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N35" s="2" t="inlineStr"/>
+      <c r="O35" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P35" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q35" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R35" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S35" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="T35" s="2" t="inlineStr">
+        <is>
+          <t>Partially Verified</t>
+        </is>
+      </c>
+      <c r="U35" s="2" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U32"/>
+  <autoFilter ref="A1:U35"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Amazon scraper checkpoint: Fashion Slippers
</commit_message>
<xml_diff>
--- a/output/Amazon_Seller_Master_Data.xlsx
+++ b/output/Amazon_Seller_Master_Data.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Amazon Sellers" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Amazon Sellers'!$A$1:$U$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Amazon Sellers'!$A$1:$U$39</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U35"/>
+  <dimension ref="A1:U39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -3606,7 +3606,7 @@
           <t>Women'S Formals</t>
         </is>
       </c>
-      <c r="B33" s="2" t="inlineStr"/>
+      <c r="B33" s="2" t="n"/>
       <c r="C33" s="3" t="n">
         <v>1</v>
       </c>
@@ -3660,7 +3660,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N33" s="2" t="inlineStr"/>
+      <c r="N33" s="2" t="n"/>
       <c r="O33" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -3703,7 +3703,7 @@
           <t>Women'S Formals</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr"/>
+      <c r="B34" s="2" t="n"/>
       <c r="C34" s="3" t="n">
         <v>2</v>
       </c>
@@ -3757,7 +3757,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N34" s="2" t="inlineStr"/>
+      <c r="N34" s="2" t="n"/>
       <c r="O34" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -3800,7 +3800,7 @@
           <t>Women'S Formals</t>
         </is>
       </c>
-      <c r="B35" s="2" t="inlineStr"/>
+      <c r="B35" s="2" t="n"/>
       <c r="C35" s="3" t="n">
         <v>3</v>
       </c>
@@ -3854,7 +3854,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N35" s="2" t="inlineStr"/>
+      <c r="N35" s="2" t="n"/>
       <c r="O35" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -3886,13 +3886,401 @@
         </is>
       </c>
       <c r="U35" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Fashion Slippers</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr"/>
+      <c r="C36" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Cocoblu Retail</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Fashion Slippers</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="inlineStr">
+        <is>
+          <t>+919217326570</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>care@cocoblu.in</t>
+        </is>
+      </c>
+      <c r="J36" s="4" t="inlineStr">
+        <is>
+          <t>29AAJCC8517E1ZH</t>
+        </is>
+      </c>
+      <c r="K36" s="4" t="inlineStr">
+        <is>
+          <t>AAJCC8517E</t>
+        </is>
+      </c>
+      <c r="L36" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M36" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="inlineStr"/>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P36" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q36" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R36" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S36" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cocoblu.in/</t>
+        </is>
+      </c>
+      <c r="T36" s="2" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="U36" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Fashion Slippers</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr"/>
+      <c r="C37" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Bata_India Ltd</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Fashion Slippers</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>+919797888868</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="J37" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K37" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L37" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M37" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N37" s="2" t="inlineStr"/>
+      <c r="O37" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P37" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q37" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R37" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S37" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="T37" s="2" t="inlineStr">
+        <is>
+          <t>Partially Verified</t>
+        </is>
+      </c>
+      <c r="U37" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Fashion Slippers</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr"/>
+      <c r="C38" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Repose Group</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Fashion Slippers</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="J38" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K38" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L38" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M38" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="inlineStr"/>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P38" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q38" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R38" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S38" s="2" t="inlineStr">
+        <is>
+          <t>https://www.vocabulary.com/</t>
+        </is>
+      </c>
+      <c r="T38" s="2" t="inlineStr">
+        <is>
+          <t>Partially Verified</t>
+        </is>
+      </c>
+      <c r="U38" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Fashion Slippers</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr"/>
+      <c r="C39" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Galaxy Fashion Point</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Fashion Slippers</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="J39" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K39" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L39" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M39" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N39" s="2" t="inlineStr"/>
+      <c r="O39" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P39" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q39" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R39" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S39" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="T39" s="2" t="inlineStr">
+        <is>
+          <t>Needs Review</t>
+        </is>
+      </c>
+      <c r="U39" s="2" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U35"/>
+  <autoFilter ref="A1:U39"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Amazon scraper checkpoint: Boys' Footwear
</commit_message>
<xml_diff>
--- a/output/Amazon_Seller_Master_Data.xlsx
+++ b/output/Amazon_Seller_Master_Data.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Amazon Sellers" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Amazon Sellers'!$A$1:$U$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Amazon Sellers'!$A$1:$U$40</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U39"/>
+  <dimension ref="A1:U40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -3897,7 +3897,7 @@
           <t>Fashion Slippers</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr"/>
+      <c r="B36" s="2" t="n"/>
       <c r="C36" s="3" t="n">
         <v>1</v>
       </c>
@@ -3951,7 +3951,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N36" s="2" t="inlineStr"/>
+      <c r="N36" s="2" t="n"/>
       <c r="O36" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -3994,7 +3994,7 @@
           <t>Fashion Slippers</t>
         </is>
       </c>
-      <c r="B37" s="2" t="inlineStr"/>
+      <c r="B37" s="2" t="n"/>
       <c r="C37" s="3" t="n">
         <v>2</v>
       </c>
@@ -4048,7 +4048,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N37" s="2" t="inlineStr"/>
+      <c r="N37" s="2" t="n"/>
       <c r="O37" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -4091,7 +4091,7 @@
           <t>Fashion Slippers</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr"/>
+      <c r="B38" s="2" t="n"/>
       <c r="C38" s="3" t="n">
         <v>3</v>
       </c>
@@ -4145,7 +4145,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N38" s="2" t="inlineStr"/>
+      <c r="N38" s="2" t="n"/>
       <c r="O38" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -4188,7 +4188,7 @@
           <t>Fashion Slippers</t>
         </is>
       </c>
-      <c r="B39" s="2" t="inlineStr"/>
+      <c r="B39" s="2" t="n"/>
       <c r="C39" s="3" t="n">
         <v>4</v>
       </c>
@@ -4242,7 +4242,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N39" s="2" t="inlineStr"/>
+      <c r="N39" s="2" t="n"/>
       <c r="O39" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -4274,13 +4274,110 @@
         </is>
       </c>
       <c r="U39" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Boys' Footwear</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr"/>
+      <c r="C40" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Viraj Ent</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Boys' Footwear</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H40" s="4" t="inlineStr">
+        <is>
+          <t>+918802812345</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>aks.niec@gmail.com</t>
+        </is>
+      </c>
+      <c r="J40" s="4" t="inlineStr">
+        <is>
+          <t>07AALFT6679B1ZT</t>
+        </is>
+      </c>
+      <c r="K40" s="4" t="inlineStr">
+        <is>
+          <t>AALFT6679B</t>
+        </is>
+      </c>
+      <c r="L40" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M40" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="inlineStr"/>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P40" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q40" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R40" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S40" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="T40" s="2" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="U40" s="2" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U39"/>
+  <autoFilter ref="A1:U40"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Amazon scraper checkpoint: Infant Footwear
</commit_message>
<xml_diff>
--- a/output/Amazon_Seller_Master_Data.xlsx
+++ b/output/Amazon_Seller_Master_Data.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Amazon Sellers" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Amazon Sellers'!$A$1:$U$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Amazon Sellers'!$A$1:$U$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U40"/>
+  <dimension ref="A1:U44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -472,7 +472,7 @@
     <col width="19" customWidth="1" min="7" max="7"/>
     <col width="17" customWidth="1" min="8" max="8"/>
     <col width="37" customWidth="1" min="9" max="9"/>
-    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="36" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
     <col width="39" customWidth="1" min="13" max="13"/>
@@ -4285,7 +4285,7 @@
           <t>Boys' Footwear</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr"/>
+      <c r="B40" s="2" t="n"/>
       <c r="C40" s="3" t="n">
         <v>1</v>
       </c>
@@ -4339,7 +4339,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N40" s="2" t="inlineStr"/>
+      <c r="N40" s="2" t="n"/>
       <c r="O40" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -4371,13 +4371,401 @@
         </is>
       </c>
       <c r="U40" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Infant Footwear</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr"/>
+      <c r="C41" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Shyamakid</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Infant Footwear</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="inlineStr">
+        <is>
+          <t>+911995071387</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>contact@shyamnamkeen.com</t>
+        </is>
+      </c>
+      <c r="J41" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K41" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L41" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M41" s="5" t="inlineStr">
+        <is>
+          <t>naga cottagecircular road dimapur in797112</t>
+        </is>
+      </c>
+      <c r="N41" s="2" t="inlineStr"/>
+      <c r="O41" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P41" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q41" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R41" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S41" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="T41" s="2" t="inlineStr">
+        <is>
+          <t>Partially Verified</t>
+        </is>
+      </c>
+      <c r="U41" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Infant Footwear</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr"/>
+      <c r="C42" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Shyama footwear</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Infant Footwear</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H42" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>contact@doctorsnutrition.com</t>
+        </is>
+      </c>
+      <c r="J42" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K42" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L42" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M42" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="inlineStr"/>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P42" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q42" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R42" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S42" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="T42" s="2" t="inlineStr">
+        <is>
+          <t>Partially Verified</t>
+        </is>
+      </c>
+      <c r="U42" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Infant Footwear</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr"/>
+      <c r="C43" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>PURESOLE</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Infant Footwear</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr">
+        <is>
+          <t>+919750419735</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>drstones@stonesfamilydental.com</t>
+        </is>
+      </c>
+      <c r="J43" s="4" t="inlineStr">
+        <is>
+          <t>27AAPCP4135R1ZL</t>
+        </is>
+      </c>
+      <c r="K43" s="4" t="inlineStr">
+        <is>
+          <t>AAPCP4135R</t>
+        </is>
+      </c>
+      <c r="L43" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M43" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N43" s="2" t="inlineStr"/>
+      <c r="O43" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P43" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q43" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R43" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S43" s="2" t="inlineStr">
+        <is>
+          <t>https://www.puresole.com/</t>
+        </is>
+      </c>
+      <c r="T43" s="2" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="U43" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Infant Footwear</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr"/>
+      <c r="C44" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>TECHSUN MART®</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Infant Footwear</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H44" s="4" t="inlineStr">
+        <is>
+          <t>+914971232026</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="J44" s="4" t="inlineStr">
+        <is>
+          <t>24AQCPL4412D1ZH; 29AQCPL4412D1Z7</t>
+        </is>
+      </c>
+      <c r="K44" s="4" t="inlineStr">
+        <is>
+          <t>AQCPL4412D</t>
+        </is>
+      </c>
+      <c r="L44" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M44" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N44" s="2" t="inlineStr"/>
+      <c r="O44" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P44" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q44" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R44" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S44" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sellerratings.com/</t>
+        </is>
+      </c>
+      <c r="T44" s="2" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="U44" s="2" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U40"/>
+  <autoFilter ref="A1:U44"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Amazon scraper checkpoint: Swimwear
</commit_message>
<xml_diff>
--- a/output/Amazon_Seller_Master_Data.xlsx
+++ b/output/Amazon_Seller_Master_Data.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Amazon Sellers" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Amazon Sellers'!$A$1:$U$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Amazon Sellers'!$A$1:$U$49</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U44"/>
+  <dimension ref="A1:U49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -4382,7 +4382,7 @@
           <t>Infant Footwear</t>
         </is>
       </c>
-      <c r="B41" s="2" t="inlineStr"/>
+      <c r="B41" s="2" t="n"/>
       <c r="C41" s="3" t="n">
         <v>1</v>
       </c>
@@ -4436,7 +4436,7 @@
           <t>naga cottagecircular road dimapur in797112</t>
         </is>
       </c>
-      <c r="N41" s="2" t="inlineStr"/>
+      <c r="N41" s="2" t="n"/>
       <c r="O41" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -4479,7 +4479,7 @@
           <t>Infant Footwear</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr"/>
+      <c r="B42" s="2" t="n"/>
       <c r="C42" s="3" t="n">
         <v>2</v>
       </c>
@@ -4533,7 +4533,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N42" s="2" t="inlineStr"/>
+      <c r="N42" s="2" t="n"/>
       <c r="O42" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -4576,7 +4576,7 @@
           <t>Infant Footwear</t>
         </is>
       </c>
-      <c r="B43" s="2" t="inlineStr"/>
+      <c r="B43" s="2" t="n"/>
       <c r="C43" s="3" t="n">
         <v>3</v>
       </c>
@@ -4630,7 +4630,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N43" s="2" t="inlineStr"/>
+      <c r="N43" s="2" t="n"/>
       <c r="O43" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -4673,7 +4673,7 @@
           <t>Infant Footwear</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr"/>
+      <c r="B44" s="2" t="n"/>
       <c r="C44" s="3" t="n">
         <v>4</v>
       </c>
@@ -4727,7 +4727,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N44" s="2" t="inlineStr"/>
+      <c r="N44" s="2" t="n"/>
       <c r="O44" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -4759,13 +4759,498 @@
         </is>
       </c>
       <c r="U44" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Swimwear</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr"/>
+      <c r="C45" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Cocoblu Retail</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Swimwear</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="inlineStr">
+        <is>
+          <t>+919217326570</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>care@cocoblu.in</t>
+        </is>
+      </c>
+      <c r="J45" s="4" t="inlineStr">
+        <is>
+          <t>29AAJCC8517E1ZH</t>
+        </is>
+      </c>
+      <c r="K45" s="4" t="inlineStr">
+        <is>
+          <t>AAJCC8517E</t>
+        </is>
+      </c>
+      <c r="L45" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M45" s="5" t="inlineStr">
+        <is>
+          <t>h. no. 51, village hauz khas, south west delhi, new delhi, in-dl, 110016, in</t>
+        </is>
+      </c>
+      <c r="N45" s="2" t="inlineStr"/>
+      <c r="O45" s="2" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="P45" s="2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="Q45" s="4" t="inlineStr">
+        <is>
+          <t>110016</t>
+        </is>
+      </c>
+      <c r="R45" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S45" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cocoblu.in/</t>
+        </is>
+      </c>
+      <c r="T45" s="2" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="U45" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Swimwear</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr"/>
+      <c r="C46" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Blissclub</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Swimwear</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H46" s="4" t="inlineStr">
+        <is>
+          <t>+919071083484</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>hi@myblissclub.in</t>
+        </is>
+      </c>
+      <c r="J46" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K46" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L46" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M46" s="5" t="inlineStr">
+        <is>
+          <t>a-143, 6th floor, sovereign corporate tower, sector- 136, noida, uttar pradesh (201305)</t>
+        </is>
+      </c>
+      <c r="N46" s="2" t="inlineStr"/>
+      <c r="O46" s="2" t="inlineStr">
+        <is>
+          <t>uttar pradesh ()</t>
+        </is>
+      </c>
+      <c r="P46" s="2" t="inlineStr">
+        <is>
+          <t>Uttar Pradesh</t>
+        </is>
+      </c>
+      <c r="Q46" s="4" t="inlineStr">
+        <is>
+          <t>201305</t>
+        </is>
+      </c>
+      <c r="R46" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S46" s="2" t="inlineStr">
+        <is>
+          <t>https://www.blissclub.com/</t>
+        </is>
+      </c>
+      <c r="T46" s="2" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="U46" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Swimwear</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr"/>
+      <c r="C47" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Neu Look Fashion</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Swimwear</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>admissions@northeastern.edu</t>
+        </is>
+      </c>
+      <c r="J47" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K47" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L47" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M47" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N47" s="2" t="inlineStr"/>
+      <c r="O47" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P47" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q47" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R47" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S47" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="T47" s="2" t="inlineStr">
+        <is>
+          <t>Partially Verified</t>
+        </is>
+      </c>
+      <c r="U47" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Swimwear</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr"/>
+      <c r="C48" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>A.P. ENTERPRISES</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Swimwear</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H48" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="J48" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K48" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L48" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M48" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N48" s="2" t="inlineStr"/>
+      <c r="O48" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P48" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q48" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R48" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S48" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="T48" s="2" t="inlineStr">
+        <is>
+          <t>Needs Review</t>
+        </is>
+      </c>
+      <c r="U48" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>Swimwear</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr"/>
+      <c r="C49" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>SANJEEV HOSIERY</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>Swimwear</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H49" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>info@nextdoor.build</t>
+        </is>
+      </c>
+      <c r="J49" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K49" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L49" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M49" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N49" s="2" t="inlineStr"/>
+      <c r="O49" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P49" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q49" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R49" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S49" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="T49" s="2" t="inlineStr">
+        <is>
+          <t>Partially Verified</t>
+        </is>
+      </c>
+      <c r="U49" s="2" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U44"/>
+  <autoFilter ref="A1:U49"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Amazon scraper checkpoint: Women'S Sports Sandals
</commit_message>
<xml_diff>
--- a/output/Amazon_Seller_Master_Data.xlsx
+++ b/output/Amazon_Seller_Master_Data.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Amazon Sellers" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Amazon Sellers'!$A$1:$U$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Amazon Sellers'!$A$1:$U$53</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U49"/>
+  <dimension ref="A1:U53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -4770,7 +4770,7 @@
           <t>Swimwear</t>
         </is>
       </c>
-      <c r="B45" s="2" t="inlineStr"/>
+      <c r="B45" s="2" t="n"/>
       <c r="C45" s="3" t="n">
         <v>1</v>
       </c>
@@ -4824,7 +4824,7 @@
           <t>h. no. 51, village hauz khas, south west delhi, new delhi, in-dl, 110016, in</t>
         </is>
       </c>
-      <c r="N45" s="2" t="inlineStr"/>
+      <c r="N45" s="2" t="n"/>
       <c r="O45" s="2" t="inlineStr">
         <is>
           <t>in</t>
@@ -4867,7 +4867,7 @@
           <t>Swimwear</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr"/>
+      <c r="B46" s="2" t="n"/>
       <c r="C46" s="3" t="n">
         <v>2</v>
       </c>
@@ -4921,7 +4921,7 @@
           <t>a-143, 6th floor, sovereign corporate tower, sector- 136, noida, uttar pradesh (201305)</t>
         </is>
       </c>
-      <c r="N46" s="2" t="inlineStr"/>
+      <c r="N46" s="2" t="n"/>
       <c r="O46" s="2" t="inlineStr">
         <is>
           <t>uttar pradesh ()</t>
@@ -4964,7 +4964,7 @@
           <t>Swimwear</t>
         </is>
       </c>
-      <c r="B47" s="2" t="inlineStr"/>
+      <c r="B47" s="2" t="n"/>
       <c r="C47" s="3" t="n">
         <v>3</v>
       </c>
@@ -5018,7 +5018,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N47" s="2" t="inlineStr"/>
+      <c r="N47" s="2" t="n"/>
       <c r="O47" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -5061,7 +5061,7 @@
           <t>Swimwear</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr"/>
+      <c r="B48" s="2" t="n"/>
       <c r="C48" s="3" t="n">
         <v>4</v>
       </c>
@@ -5115,7 +5115,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N48" s="2" t="inlineStr"/>
+      <c r="N48" s="2" t="n"/>
       <c r="O48" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -5158,7 +5158,7 @@
           <t>Swimwear</t>
         </is>
       </c>
-      <c r="B49" s="2" t="inlineStr"/>
+      <c r="B49" s="2" t="n"/>
       <c r="C49" s="3" t="n">
         <v>5</v>
       </c>
@@ -5212,7 +5212,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N49" s="2" t="inlineStr"/>
+      <c r="N49" s="2" t="n"/>
       <c r="O49" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -5244,13 +5244,401 @@
         </is>
       </c>
       <c r="U49" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Women'S Sports Sandals</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr"/>
+      <c r="C50" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Campusactivewear</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Women'S Sports Sandals</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H50" s="4" t="inlineStr">
+        <is>
+          <t>+919667706012</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>compliance@campusshoes.com</t>
+        </is>
+      </c>
+      <c r="J50" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K50" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L50" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M50" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N50" s="2" t="inlineStr"/>
+      <c r="O50" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P50" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q50" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R50" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S50" s="2" t="inlineStr">
+        <is>
+          <t>https://www.campusactivewear.com/</t>
+        </is>
+      </c>
+      <c r="T50" s="2" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="U50" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Women'S Sports Sandals</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr"/>
+      <c r="C51" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Cocoblu Retail</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>Women'S Sports Sandals</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H51" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="J51" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K51" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L51" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M51" s="5" t="inlineStr">
+        <is>
+          <t>1722 atlantic ave a, atlantic city, nj 08401 😻hey</t>
+        </is>
+      </c>
+      <c r="N51" s="2" t="inlineStr"/>
+      <c r="O51" s="2" t="inlineStr">
+        <is>
+          <t>atlantic city</t>
+        </is>
+      </c>
+      <c r="P51" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q51" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R51" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S51" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="T51" s="2" t="inlineStr">
+        <is>
+          <t>Partially Verified</t>
+        </is>
+      </c>
+      <c r="U51" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>Women'S Sports Sandals</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr"/>
+      <c r="C52" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Bata_India Ltd</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>Women'S Sports Sandals</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H52" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="J52" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K52" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L52" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M52" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N52" s="2" t="inlineStr"/>
+      <c r="O52" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P52" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q52" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R52" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S52" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="T52" s="2" t="inlineStr">
+        <is>
+          <t>Needs Review</t>
+        </is>
+      </c>
+      <c r="U52" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>Women'S Sports Sandals</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr"/>
+      <c r="C53" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Yoho Lifestyle</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>Women'S Sports Sandals</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H53" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>support@tradmap.com</t>
+        </is>
+      </c>
+      <c r="J53" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K53" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L53" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M53" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N53" s="2" t="inlineStr"/>
+      <c r="O53" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P53" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q53" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R53" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S53" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="T53" s="2" t="inlineStr">
+        <is>
+          <t>Partially Verified</t>
+        </is>
+      </c>
+      <c r="U53" s="2" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U49"/>
+  <autoFilter ref="A1:U53"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Amazon scraper checkpoint: School Uniforms
</commit_message>
<xml_diff>
--- a/output/Amazon_Seller_Master_Data.xlsx
+++ b/output/Amazon_Seller_Master_Data.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Amazon Sellers" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Amazon Sellers'!$A$1:$U$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Amazon Sellers'!$A$1:$U$56</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U53"/>
+  <dimension ref="A1:U56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -5546,7 +5546,7 @@
           <t>Boys' Footwear</t>
         </is>
       </c>
-      <c r="B53" s="2" t="inlineStr"/>
+      <c r="B53" s="2" t="n"/>
       <c r="C53" s="3" t="n">
         <v>1</v>
       </c>
@@ -5600,7 +5600,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N53" s="2" t="inlineStr"/>
+      <c r="N53" s="2" t="n"/>
       <c r="O53" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -5632,13 +5632,304 @@
         </is>
       </c>
       <c r="U53" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>School Uniforms</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr"/>
+      <c r="C54" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>PUPPETNX</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>School Uniforms</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H54" s="4" t="inlineStr">
+        <is>
+          <t>+919825985840</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>puppetnx1986@gmail.com</t>
+        </is>
+      </c>
+      <c r="J54" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K54" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L54" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M54" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N54" s="2" t="inlineStr"/>
+      <c r="O54" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P54" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q54" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R54" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.puppetnx.com/</t>
+        </is>
+      </c>
+      <c r="T54" s="2" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="U54" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>School Uniforms</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr"/>
+      <c r="C55" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>HORN Dark K</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>School Uniforms</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H55" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="J55" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K55" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L55" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M55" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N55" s="2" t="inlineStr"/>
+      <c r="O55" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P55" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q55" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R55" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S55" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="T55" s="2" t="inlineStr">
+        <is>
+          <t>Needs Review</t>
+        </is>
+      </c>
+      <c r="U55" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>School Uniforms</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr"/>
+      <c r="C56" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>MODI AGENCY</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>School Uniforms</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H56" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="J56" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K56" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L56" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M56" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N56" s="2" t="inlineStr"/>
+      <c r="O56" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P56" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q56" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R56" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S56" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="T56" s="2" t="inlineStr">
+        <is>
+          <t>Partially Verified</t>
+        </is>
+      </c>
+      <c r="U56" s="2" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U53"/>
+  <autoFilter ref="A1:U56"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Amazon scraper checkpoint: Dungarees
</commit_message>
<xml_diff>
--- a/output/Amazon_Seller_Master_Data.xlsx
+++ b/output/Amazon_Seller_Master_Data.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Amazon Sellers" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Amazon Sellers'!$A$1:$U$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Amazon Sellers'!$A$1:$U$62</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U56"/>
+  <dimension ref="A1:U62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -471,7 +471,7 @@
     <col width="31" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
     <col width="17" customWidth="1" min="8" max="8"/>
-    <col width="37" customWidth="1" min="9" max="9"/>
+    <col width="49" customWidth="1" min="9" max="9"/>
     <col width="36" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
@@ -5643,7 +5643,7 @@
           <t>School Uniforms</t>
         </is>
       </c>
-      <c r="B54" s="2" t="inlineStr"/>
+      <c r="B54" s="2" t="n"/>
       <c r="C54" s="3" t="n">
         <v>1</v>
       </c>
@@ -5697,7 +5697,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N54" s="2" t="inlineStr"/>
+      <c r="N54" s="2" t="n"/>
       <c r="O54" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -5740,7 +5740,7 @@
           <t>School Uniforms</t>
         </is>
       </c>
-      <c r="B55" s="2" t="inlineStr"/>
+      <c r="B55" s="2" t="n"/>
       <c r="C55" s="3" t="n">
         <v>2</v>
       </c>
@@ -5794,7 +5794,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N55" s="2" t="inlineStr"/>
+      <c r="N55" s="2" t="n"/>
       <c r="O55" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -5837,7 +5837,7 @@
           <t>School Uniforms</t>
         </is>
       </c>
-      <c r="B56" s="2" t="inlineStr"/>
+      <c r="B56" s="2" t="n"/>
       <c r="C56" s="3" t="n">
         <v>3</v>
       </c>
@@ -5891,7 +5891,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N56" s="2" t="inlineStr"/>
+      <c r="N56" s="2" t="n"/>
       <c r="O56" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -5923,13 +5923,595 @@
         </is>
       </c>
       <c r="U56" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>Dungarees</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr"/>
+      <c r="C57" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>KiddoPanti</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>Dungarees</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H57" s="4" t="inlineStr">
+        <is>
+          <t>+919972924523</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>customercare@kiddopanti.com</t>
+        </is>
+      </c>
+      <c r="J57" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K57" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L57" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M57" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N57" s="2" t="inlineStr"/>
+      <c r="O57" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P57" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q57" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R57" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S57" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kiddopanti.com/</t>
+        </is>
+      </c>
+      <c r="T57" s="2" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="U57" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Dungarees</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr"/>
+      <c r="C58" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>Cocoblu Retail</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>Dungarees</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H58" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>support@touchofmodern.com</t>
+        </is>
+      </c>
+      <c r="J58" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K58" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L58" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M58" s="5" t="inlineStr">
+        <is>
+          <t>by signing up, you agree to our terms of service and privacy policy. you may unsubscribe at any time.</t>
+        </is>
+      </c>
+      <c r="N58" s="2" t="inlineStr"/>
+      <c r="O58" s="2" t="inlineStr">
+        <is>
+          <t>by signing up</t>
+        </is>
+      </c>
+      <c r="P58" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q58" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R58" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S58" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="T58" s="2" t="inlineStr">
+        <is>
+          <t>Partially Verified</t>
+        </is>
+      </c>
+      <c r="U58" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Dungarees</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr"/>
+      <c r="C59" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>Chase Labs</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>Dungarees</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H59" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="J59" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K59" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L59" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M59" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N59" s="2" t="inlineStr"/>
+      <c r="O59" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P59" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q59" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R59" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S59" s="2" t="inlineStr">
+        <is>
+          <t>https://www.chaselabs.com/</t>
+        </is>
+      </c>
+      <c r="T59" s="2" t="inlineStr">
+        <is>
+          <t>Partially Verified</t>
+        </is>
+      </c>
+      <c r="U59" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Dungarees</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr"/>
+      <c r="C60" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>KIVIRO</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>Dungarees</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H60" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="J60" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K60" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L60" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M60" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N60" s="2" t="inlineStr"/>
+      <c r="O60" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P60" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q60" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R60" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S60" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kiviro.in/</t>
+        </is>
+      </c>
+      <c r="T60" s="2" t="inlineStr">
+        <is>
+          <t>Partially Verified</t>
+        </is>
+      </c>
+      <c r="U60" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>Dungarees</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr"/>
+      <c r="C61" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>KARISHMA FASHIONS</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>Dungarees</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H61" s="4" t="inlineStr">
+        <is>
+          <t>+916404199475</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>aclaracionesyrectificaciones@elespectador.com</t>
+        </is>
+      </c>
+      <c r="J61" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K61" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L61" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M61" s="5" t="inlineStr">
+        <is>
+          <t>128 s. washington st.</t>
+        </is>
+      </c>
+      <c r="N61" s="2" t="inlineStr"/>
+      <c r="O61" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P61" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q61" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R61" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S61" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stylestone.in/</t>
+        </is>
+      </c>
+      <c r="T61" s="2" t="inlineStr">
+        <is>
+          <t>Partially Verified</t>
+        </is>
+      </c>
+      <c r="U61" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>Dungarees</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr"/>
+      <c r="C62" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>Indicreate Designs</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>Dungarees</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H62" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>dro@osc.state.ny.us</t>
+        </is>
+      </c>
+      <c r="J62" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K62" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L62" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M62" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N62" s="2" t="inlineStr"/>
+      <c r="O62" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P62" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q62" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R62" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S62" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="T62" s="2" t="inlineStr">
+        <is>
+          <t>Partially Verified</t>
+        </is>
+      </c>
+      <c r="U62" s="2" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U56"/>
+  <autoFilter ref="A1:U62"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Amazon scraper checkpoint: Tops, T-Shirts & Shirts
</commit_message>
<xml_diff>
--- a/output/Amazon_Seller_Master_Data.xlsx
+++ b/output/Amazon_Seller_Master_Data.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Amazon Sellers" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Amazon Sellers'!$A$1:$U$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Amazon Sellers'!$A$1:$U$64</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U62"/>
+  <dimension ref="A1:U64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -469,7 +469,7 @@
     <col width="38" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="31" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="17" customWidth="1" min="8" max="8"/>
     <col width="49" customWidth="1" min="9" max="9"/>
     <col width="36" customWidth="1" min="10" max="10"/>
@@ -5934,7 +5934,7 @@
           <t>Dungarees</t>
         </is>
       </c>
-      <c r="B57" s="2" t="inlineStr"/>
+      <c r="B57" s="2" t="n"/>
       <c r="C57" s="3" t="n">
         <v>1</v>
       </c>
@@ -5988,7 +5988,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N57" s="2" t="inlineStr"/>
+      <c r="N57" s="2" t="n"/>
       <c r="O57" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -6031,7 +6031,7 @@
           <t>Dungarees</t>
         </is>
       </c>
-      <c r="B58" s="2" t="inlineStr"/>
+      <c r="B58" s="2" t="n"/>
       <c r="C58" s="3" t="n">
         <v>2</v>
       </c>
@@ -6085,7 +6085,7 @@
           <t>by signing up, you agree to our terms of service and privacy policy. you may unsubscribe at any time.</t>
         </is>
       </c>
-      <c r="N58" s="2" t="inlineStr"/>
+      <c r="N58" s="2" t="n"/>
       <c r="O58" s="2" t="inlineStr">
         <is>
           <t>by signing up</t>
@@ -6128,7 +6128,7 @@
           <t>Dungarees</t>
         </is>
       </c>
-      <c r="B59" s="2" t="inlineStr"/>
+      <c r="B59" s="2" t="n"/>
       <c r="C59" s="3" t="n">
         <v>3</v>
       </c>
@@ -6182,7 +6182,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N59" s="2" t="inlineStr"/>
+      <c r="N59" s="2" t="n"/>
       <c r="O59" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -6225,7 +6225,7 @@
           <t>Dungarees</t>
         </is>
       </c>
-      <c r="B60" s="2" t="inlineStr"/>
+      <c r="B60" s="2" t="n"/>
       <c r="C60" s="3" t="n">
         <v>4</v>
       </c>
@@ -6279,7 +6279,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N60" s="2" t="inlineStr"/>
+      <c r="N60" s="2" t="n"/>
       <c r="O60" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -6322,7 +6322,7 @@
           <t>Dungarees</t>
         </is>
       </c>
-      <c r="B61" s="2" t="inlineStr"/>
+      <c r="B61" s="2" t="n"/>
       <c r="C61" s="3" t="n">
         <v>5</v>
       </c>
@@ -6376,7 +6376,7 @@
           <t>128 s. washington st.</t>
         </is>
       </c>
-      <c r="N61" s="2" t="inlineStr"/>
+      <c r="N61" s="2" t="n"/>
       <c r="O61" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -6419,7 +6419,7 @@
           <t>Dungarees</t>
         </is>
       </c>
-      <c r="B62" s="2" t="inlineStr"/>
+      <c r="B62" s="2" t="n"/>
       <c r="C62" s="3" t="n">
         <v>6</v>
       </c>
@@ -6473,7 +6473,7 @@
           <t>Not Found</t>
         </is>
       </c>
-      <c r="N62" s="2" t="inlineStr"/>
+      <c r="N62" s="2" t="n"/>
       <c r="O62" s="2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -6505,13 +6505,207 @@
         </is>
       </c>
       <c r="U62" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>Tops, T-Shirts &amp; Shirts</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr"/>
+      <c r="C63" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>KARTBIN ONLINE SERVICES PVT LTD</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>Tops, T-Shirts &amp; Shirts</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H63" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>help@firecrawl.com</t>
+        </is>
+      </c>
+      <c r="J63" s="4" t="inlineStr">
+        <is>
+          <t>06AAFCK5111Q1ZC</t>
+        </is>
+      </c>
+      <c r="K63" s="4" t="inlineStr">
+        <is>
+          <t>AAFCK5111Q</t>
+        </is>
+      </c>
+      <c r="L63" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M63" s="5" t="inlineStr">
+        <is>
+          <t>p.o. box 145496, cincinnati, oh 45250-5496. © 2026 cincinnati financial corporation.</t>
+        </is>
+      </c>
+      <c r="N63" s="2" t="inlineStr"/>
+      <c r="O63" s="2" t="inlineStr">
+        <is>
+          <t>cincinnati</t>
+        </is>
+      </c>
+      <c r="P63" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q63" s="4" t="inlineStr">
+        <is>
+          <t>145496</t>
+        </is>
+      </c>
+      <c r="R63" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S63" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="T63" s="2" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="U63" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>Tops, T-Shirts &amp; Shirts</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr"/>
+      <c r="C64" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Frost Clothings</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>Tops, T-Shirts &amp; Shirts</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>townsquare media</t>
+        </is>
+      </c>
+      <c r="H64" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>a.murray@bep-la.com</t>
+        </is>
+      </c>
+      <c r="J64" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="K64" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="L64" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M64" s="5" t="inlineStr">
+        <is>
+          <t>one city center, portland, me 04101</t>
+        </is>
+      </c>
+      <c r="N64" s="2" t="inlineStr"/>
+      <c r="O64" s="2" t="inlineStr">
+        <is>
+          <t>portland</t>
+        </is>
+      </c>
+      <c r="P64" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q64" s="4" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R64" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S64" s="2" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="T64" s="2" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="U64" s="2" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U62"/>
+  <autoFilter ref="A1:U64"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>